<commit_message>
Pipeline run: update roster and extractions
</commit_message>
<xml_diff>
--- a/data/final/ir_extraction.xlsx
+++ b/data/final/ir_extraction.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BZ27"/>
+  <dimension ref="A1:CA27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -811,6 +811,11 @@
           <t>Supplementary material</t>
         </is>
       </c>
+      <c r="CA1" s="1" t="inlineStr">
+        <is>
+          <t>Data quality flag</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1191,6 +1196,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1571,6 +1581,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1951,6 +1966,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2331,6 +2351,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA5" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2705,6 +2730,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA6" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3079,6 +3109,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3453,6 +3488,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3827,6 +3867,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4201,6 +4246,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA10" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4575,6 +4625,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4949,6 +5004,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5323,6 +5383,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5697,6 +5762,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA14" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6071,6 +6141,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA15" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6445,6 +6520,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6819,6 +6899,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA17" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7199,6 +7284,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA18" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7579,6 +7669,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA19" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7953,6 +8048,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA20" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -8323,6 +8423,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA21" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -8693,6 +8798,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA22" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -9071,6 +9181,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA23" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -9449,6 +9564,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA24" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -9827,6 +9947,11 @@
           <t>NA</t>
         </is>
       </c>
+      <c r="CA25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -10009,21 +10134,17 @@
       <c r="AL26" t="n">
         <v>75</v>
       </c>
-      <c r="AM26" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AN26" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+      <c r="AM26" t="n">
+        <v>5</v>
+      </c>
+      <c r="AN26" t="n">
+        <v>70</v>
       </c>
       <c r="AO26" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.0667</v>
       </c>
       <c r="AP26" t="n">
-        <v>0.93</v>
+        <v>0.9333</v>
       </c>
       <c r="AQ26" t="inlineStr">
         <is>
@@ -10172,7 +10293,7 @@
       </c>
       <c r="BT26" t="inlineStr">
         <is>
-          <t>no (reported mortality only)</t>
+          <t>derived (reported % x n)</t>
         </is>
       </c>
       <c r="BU26" t="inlineStr">
@@ -10203,6 +10324,11 @@
       <c r="BZ26" t="inlineStr">
         <is>
           <t>NA</t>
+        </is>
+      </c>
+      <c r="CA26" t="inlineStr">
+        <is>
+          <t>dead/surviving counts derived in code from reported % x number exposed</t>
         </is>
       </c>
     </row>
@@ -10387,21 +10513,17 @@
       <c r="AL27" t="n">
         <v>90</v>
       </c>
-      <c r="AM27" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AN27" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+      <c r="AM27" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN27" t="n">
+        <v>87</v>
       </c>
       <c r="AO27" t="n">
-        <v>0.03</v>
+        <v>0.0333</v>
       </c>
       <c r="AP27" t="n">
-        <v>0.97</v>
+        <v>0.9667</v>
       </c>
       <c r="AQ27" t="inlineStr">
         <is>
@@ -10550,7 +10672,7 @@
       </c>
       <c r="BT27" t="inlineStr">
         <is>
-          <t>no (reported mortality only)</t>
+          <t>derived (reported % x n)</t>
         </is>
       </c>
       <c r="BU27" t="inlineStr">
@@ -10581,6 +10703,11 @@
       <c r="BZ27" t="inlineStr">
         <is>
           <t>NA</t>
+        </is>
+      </c>
+      <c r="CA27" t="inlineStr">
+        <is>
+          <t>dead/surviving counts derived in code from reported % x number exposed</t>
         </is>
       </c>
     </row>

</xml_diff>